<commit_message>
Added Task 1 copies and Task 3 initials based off Tast 1
</commit_message>
<xml_diff>
--- a/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
+++ b/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/smtros022_myuct_ac_za/Documents/Fourth Year/Sem 2/EEE3096S/EEE3096S Git Repo SMTROS022/EEE3096S SMTROS022 Pracs/Prac 3/Misc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44CA6F7B-6711-4A77-BC51-BECC1736D54F}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CBF68F7-43B0-4D0F-8A88-F4B94C2AF643}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB21F44C-0F24-4ECD-93E7-EFB15482C059}"/>
   </bookViews>
@@ -1039,12 +1039,24 @@
       <c r="M12" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="4"/>
-      <c r="S12" s="4"/>
+      <c r="N12" s="4">
+        <v>429346</v>
+      </c>
+      <c r="O12" s="4">
+        <v>21874</v>
+      </c>
+      <c r="P12" s="4">
+        <v>968024</v>
+      </c>
+      <c r="Q12" s="4">
+        <v>48764</v>
+      </c>
+      <c r="R12" s="4">
+        <v>1858360</v>
+      </c>
+      <c r="S12" s="4">
+        <v>93198</v>
+      </c>
       <c r="T12" s="4"/>
       <c r="U12" s="4"/>
       <c r="V12" s="4"/>
@@ -1087,12 +1099,24 @@
       <c r="M13" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="N13" s="6"/>
-      <c r="O13" s="6"/>
-      <c r="P13" s="6"/>
-      <c r="Q13" s="6"/>
-      <c r="R13" s="6"/>
-      <c r="S13" s="6"/>
+      <c r="N13" s="6">
+        <v>669809</v>
+      </c>
+      <c r="O13" s="6">
+        <v>34169</v>
+      </c>
+      <c r="P13" s="6">
+        <v>1510353</v>
+      </c>
+      <c r="Q13" s="6">
+        <v>76225</v>
+      </c>
+      <c r="R13" s="6">
+        <v>2899477</v>
+      </c>
+      <c r="S13" s="6">
+        <v>145712</v>
+      </c>
       <c r="T13" s="6"/>
       <c r="U13" s="6"/>
       <c r="V13" s="6"/>
@@ -1135,12 +1159,24 @@
       <c r="M14" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="4"/>
-      <c r="S14" s="4"/>
+      <c r="N14" s="4">
+        <v>966227</v>
+      </c>
+      <c r="O14" s="4">
+        <v>49327</v>
+      </c>
+      <c r="P14" s="4">
+        <v>2180459</v>
+      </c>
+      <c r="Q14" s="4">
+        <v>110117</v>
+      </c>
+      <c r="R14" s="4">
+        <v>4184222</v>
+      </c>
+      <c r="S14" s="4">
+        <v>210418</v>
+      </c>
       <c r="T14" s="4"/>
       <c r="U14" s="4"/>
       <c r="V14" s="4"/>
@@ -1183,10 +1219,18 @@
       <c r="M15" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="N15" s="6"/>
-      <c r="O15" s="6"/>
-      <c r="P15" s="6"/>
-      <c r="Q15" s="6"/>
+      <c r="N15" s="6">
+        <v>1315085</v>
+      </c>
+      <c r="O15" s="6">
+        <v>67163</v>
+      </c>
+      <c r="P15" s="6">
+        <v>2963856</v>
+      </c>
+      <c r="Q15" s="6">
+        <v>149757</v>
+      </c>
       <c r="R15" s="6"/>
       <c r="S15" s="6"/>
       <c r="T15" s="6"/>
@@ -1231,10 +1275,18 @@
       <c r="M16" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
+      <c r="N16" s="4">
+        <v>1715815</v>
+      </c>
+      <c r="O16" s="4">
+        <v>87696</v>
+      </c>
+      <c r="P16" s="4">
+        <v>3873054</v>
+      </c>
+      <c r="Q16" s="4">
+        <v>195829</v>
+      </c>
       <c r="R16" s="4"/>
       <c r="S16" s="4"/>
       <c r="T16" s="4"/>

</xml_diff>

<commit_message>
Task 3 initial edits, incorporating Time Ex
</commit_message>
<xml_diff>
--- a/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
+++ b/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/smtros022_myuct_ac_za/Documents/Fourth Year/Sem 2/EEE3096S/EEE3096S Git Repo SMTROS022/EEE3096S SMTROS022 Pracs/Prac 3/Misc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CBF68F7-43B0-4D0F-8A88-F4B94C2AF643}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C613415-518B-4512-A505-4969D2B4FC91}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB21F44C-0F24-4ECD-93E7-EFB15482C059}"/>
   </bookViews>
@@ -1057,8 +1057,12 @@
       <c r="S12" s="4">
         <v>93198</v>
       </c>
-      <c r="T12" s="4"/>
-      <c r="U12" s="4"/>
+      <c r="T12" s="4">
+        <v>2745724</v>
+      </c>
+      <c r="U12" s="4">
+        <v>137482</v>
+      </c>
       <c r="V12" s="4"/>
       <c r="W12" s="4"/>
     </row>
@@ -1117,8 +1121,12 @@
       <c r="S13" s="6">
         <v>145712</v>
       </c>
-      <c r="T13" s="6"/>
-      <c r="U13" s="6"/>
+      <c r="T13" s="6">
+        <v>4281267</v>
+      </c>
+      <c r="U13" s="6">
+        <v>214830</v>
+      </c>
       <c r="V13" s="6"/>
       <c r="W13" s="6"/>
     </row>
@@ -1177,8 +1185,12 @@
       <c r="S14" s="4">
         <v>210418</v>
       </c>
-      <c r="T14" s="4"/>
-      <c r="U14" s="4"/>
+      <c r="T14" s="4">
+        <v>6180826</v>
+      </c>
+      <c r="U14" s="4">
+        <v>310353</v>
+      </c>
       <c r="V14" s="4"/>
       <c r="W14" s="4"/>
     </row>
@@ -1231,10 +1243,18 @@
       <c r="Q15" s="6">
         <v>149757</v>
       </c>
-      <c r="R15" s="6"/>
-      <c r="S15" s="6"/>
-      <c r="T15" s="6"/>
-      <c r="U15" s="6"/>
+      <c r="R15" s="6">
+        <v>5685832</v>
+      </c>
+      <c r="S15" s="6">
+        <v>286090</v>
+      </c>
+      <c r="T15" s="6">
+        <v>8399750</v>
+      </c>
+      <c r="U15" s="6">
+        <v>422011</v>
+      </c>
       <c r="V15" s="6"/>
       <c r="W15" s="6"/>
     </row>
@@ -1287,10 +1307,18 @@
       <c r="Q16" s="4">
         <v>195829</v>
       </c>
-      <c r="R16" s="4"/>
-      <c r="S16" s="4"/>
-      <c r="T16" s="4"/>
-      <c r="U16" s="4"/>
+      <c r="R16" s="4">
+        <v>7434783</v>
+      </c>
+      <c r="S16" s="4">
+        <v>374326</v>
+      </c>
+      <c r="T16" s="4">
+        <v>10985970</v>
+      </c>
+      <c r="U16" s="4">
+        <v>552290</v>
+      </c>
       <c r="V16" s="4"/>
       <c r="W16" s="4"/>
     </row>

</xml_diff>

<commit_message>
Task 4 initial push based off task 3
</commit_message>
<xml_diff>
--- a/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
+++ b/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/smtros022_myuct_ac_za/Documents/Fourth Year/Sem 2/EEE3096S/EEE3096S Git Repo SMTROS022/EEE3096S SMTROS022 Pracs/Prac 3/Misc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="118" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{387BA547-A2C0-4A0E-8513-80FE10D339B1}"/>
+  <xr:revisionPtr revIDLastSave="132" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE692FE3-330D-483C-AA1A-1DD9B98B2E7B}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB21F44C-0F24-4ECD-93E7-EFB15482C059}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="31">
   <si>
     <t>Resolution</t>
   </si>
@@ -108,6 +108,27 @@
   </si>
   <si>
     <t>747.308899</t>
+  </si>
+  <si>
+    <t>11248.1934</t>
+  </si>
+  <si>
+    <t>11263.9375</t>
+  </si>
+  <si>
+    <t>11243.1982</t>
+  </si>
+  <si>
+    <t>11243.0596</t>
+  </si>
+  <si>
+    <t>11254.917</t>
+  </si>
+  <si>
+    <t>Task 3 F4</t>
+  </si>
+  <si>
+    <t>Task 3 F0</t>
   </si>
 </sst>
 </file>
@@ -1369,10 +1390,10 @@
     </row>
     <row r="18" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="H18" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:12" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
@@ -1417,8 +1438,12 @@
       <c r="C20" s="4">
         <v>1456</v>
       </c>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
+      <c r="D20" s="4">
+        <v>174790741</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>24</v>
+      </c>
       <c r="H20" s="3" t="s">
         <v>7</v>
       </c>
@@ -1445,8 +1470,12 @@
       <c r="C21" s="6">
         <v>2272</v>
       </c>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
+      <c r="D21" s="6">
+        <v>272728812</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>25</v>
+      </c>
       <c r="H21" s="5" t="s">
         <v>8</v>
       </c>
@@ -1473,8 +1502,12 @@
       <c r="C22" s="4">
         <v>3278</v>
       </c>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
+      <c r="D22" s="4">
+        <v>393453876</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>26</v>
+      </c>
       <c r="H22" s="3" t="s">
         <v>9</v>
       </c>
@@ -1501,8 +1534,12 @@
       <c r="C23" s="6">
         <v>4462</v>
       </c>
-      <c r="D23" s="6"/>
-      <c r="E23" s="6"/>
+      <c r="D23" s="6">
+        <v>535541064</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>27</v>
+      </c>
       <c r="H23" s="5" t="s">
         <v>10</v>
       </c>
@@ -1529,8 +1566,12 @@
       <c r="C24" s="4">
         <v>5822</v>
       </c>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
+      <c r="D24" s="4">
+        <v>698745311</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>28</v>
+      </c>
       <c r="H24" s="3" t="s">
         <v>11</v>
       </c>

</xml_diff>

<commit_message>
Task 5 Complete and Task 7 Initial based on Task 1
</commit_message>
<xml_diff>
--- a/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
+++ b/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/smtros022_myuct_ac_za/Documents/Fourth Year/Sem 2/EEE3096S/EEE3096S Git Repo SMTROS022/EEE3096S SMTROS022 Pracs/Prac 3/Misc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="409" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BC05B23D-85A6-4021-B907-02E0DCE0A662}"/>
+  <xr:revisionPtr revIDLastSave="455" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{108138AB-7840-4B11-A8D9-11C7150FFF91}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB21F44C-0F24-4ECD-93E7-EFB15482C059}"/>
+    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB21F44C-0F24-4ECD-93E7-EFB15482C059}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="68">
   <si>
     <t>Resolution</t>
   </si>
@@ -228,6 +228,18 @@
   </si>
   <si>
     <t>Task 4 F0</t>
+  </si>
+  <si>
+    <t>Checksum (Float)</t>
+  </si>
+  <si>
+    <t>Time (ms) (Float)</t>
+  </si>
+  <si>
+    <t>Task 5 FPU</t>
+  </si>
+  <si>
+    <t>Task 5 NO FPU</t>
   </si>
 </sst>
 </file>
@@ -740,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D06E983-B581-4B51-A88B-00887F6C9E77}">
-  <dimension ref="A1:W38"/>
+  <dimension ref="A1:W54"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" customWidth="1"/>
@@ -750,7 +762,7 @@
     <col min="6" max="6" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
@@ -2147,6 +2159,292 @@
         <v>40</v>
       </c>
     </row>
+    <row r="40" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" s="4">
+        <v>429346</v>
+      </c>
+      <c r="C42" s="4">
+        <v>1456</v>
+      </c>
+      <c r="D42" s="4">
+        <v>429364</v>
+      </c>
+      <c r="E42" s="4">
+        <v>77</v>
+      </c>
+      <c r="F42" s="4">
+        <v>429384</v>
+      </c>
+      <c r="G42" s="4">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B43" s="6">
+        <v>669809</v>
+      </c>
+      <c r="C43" s="6">
+        <v>2272</v>
+      </c>
+      <c r="D43" s="6">
+        <v>669834</v>
+      </c>
+      <c r="E43" s="6">
+        <v>120</v>
+      </c>
+      <c r="F43" s="6">
+        <v>669829</v>
+      </c>
+      <c r="G43" s="6">
+        <v>4235</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B44" s="4">
+        <v>966227</v>
+      </c>
+      <c r="C44" s="4">
+        <v>3278</v>
+      </c>
+      <c r="D44" s="4">
+        <v>966071</v>
+      </c>
+      <c r="E44" s="4">
+        <v>174</v>
+      </c>
+      <c r="F44" s="4">
+        <v>966024</v>
+      </c>
+      <c r="G44" s="4">
+        <v>6093</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B45" s="6">
+        <v>1315085</v>
+      </c>
+      <c r="C45" s="6">
+        <v>4462</v>
+      </c>
+      <c r="D45" s="6">
+        <v>1315044</v>
+      </c>
+      <c r="E45" s="6">
+        <v>237</v>
+      </c>
+      <c r="F45" s="6">
+        <v>1314999</v>
+      </c>
+      <c r="G45" s="6">
+        <v>8328</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" s="4">
+        <v>1715815</v>
+      </c>
+      <c r="C46" s="4">
+        <v>5822</v>
+      </c>
+      <c r="D46" s="4">
+        <v>1715808</v>
+      </c>
+      <c r="E46" s="4">
+        <v>309</v>
+      </c>
+      <c r="F46" s="4">
+        <v>1715812</v>
+      </c>
+      <c r="G46" s="4">
+        <v>10598</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B50" s="4">
+        <v>429346</v>
+      </c>
+      <c r="C50" s="4">
+        <v>1456</v>
+      </c>
+      <c r="D50" s="4">
+        <v>429364</v>
+      </c>
+      <c r="E50" s="4">
+        <v>1608</v>
+      </c>
+      <c r="F50" s="4">
+        <v>429384</v>
+      </c>
+      <c r="G50" s="4">
+        <v>2645</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B51" s="6">
+        <v>669809</v>
+      </c>
+      <c r="C51" s="6">
+        <v>2272</v>
+      </c>
+      <c r="D51" s="6">
+        <v>669834</v>
+      </c>
+      <c r="E51" s="6">
+        <v>2535</v>
+      </c>
+      <c r="F51" s="6">
+        <v>669829</v>
+      </c>
+      <c r="G51" s="6">
+        <v>4238</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B52" s="4">
+        <v>966227</v>
+      </c>
+      <c r="C52" s="4">
+        <v>3278</v>
+      </c>
+      <c r="D52" s="4">
+        <v>966071</v>
+      </c>
+      <c r="E52" s="4">
+        <v>3655</v>
+      </c>
+      <c r="F52" s="4">
+        <v>966024</v>
+      </c>
+      <c r="G52" s="4">
+        <v>6096</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B53" s="6">
+        <v>1315085</v>
+      </c>
+      <c r="C53" s="6">
+        <v>4462</v>
+      </c>
+      <c r="D53" s="6">
+        <v>1315044</v>
+      </c>
+      <c r="E53" s="6">
+        <v>4980</v>
+      </c>
+      <c r="F53" s="6">
+        <v>1314999</v>
+      </c>
+      <c r="G53" s="6">
+        <v>8334</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B54" s="4">
+        <v>1715815</v>
+      </c>
+      <c r="C54" s="4">
+        <v>5822</v>
+      </c>
+      <c r="D54" s="4">
+        <v>1715808</v>
+      </c>
+      <c r="E54" s="4">
+        <v>6443</v>
+      </c>
+      <c r="F54" s="4">
+        <v>1715812</v>
+      </c>
+      <c r="G54" s="4">
+        <v>10600</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="P10:Q10"/>

</xml_diff>

<commit_message>
Final Pushes for Prac 3
</commit_message>
<xml_diff>
--- a/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
+++ b/EEE3096S SMTROS022 Pracs/Prac 3/Misc/Raw Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uctcloud-my.sharepoint.com/personal/smtros022_myuct_ac_za/Documents/Fourth Year/Sem 2/EEE3096S/EEE3096S Git Repo SMTROS022/EEE3096S SMTROS022 Pracs/Prac 3/Misc/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="526" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E1E7B5FE-6F95-470D-AC14-5E0A326E1CF5}"/>
+  <xr:revisionPtr revIDLastSave="539" documentId="8_{C64EA8E1-BEFA-49D1-BF1E-9A3345DDF2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2710EBC-2045-4236-AAF8-1A9A5BB21096}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DB21F44C-0F24-4ECD-93E7-EFB15482C059}"/>
+    <workbookView xWindow="-21504" yWindow="0" windowWidth="21600" windowHeight="11232" xr2:uid="{DB21F44C-0F24-4ECD-93E7-EFB15482C059}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -391,7 +391,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -411,17 +411,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -777,13 +774,10 @@
     <col min="12" max="12" width="13.42578125" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="12.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="15" width="12" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="33.140625" customWidth="1"/>
+    <col min="16" max="16" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.85546875" customWidth="1"/>
+    <col min="19" max="23" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1070,46 +1064,46 @@
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="7">
         <v>100</v>
       </c>
       <c r="C10" s="8"/>
-      <c r="D10" s="7">
+      <c r="D10" s="9">
         <v>250</v>
       </c>
       <c r="E10" s="8"/>
-      <c r="F10" s="7">
+      <c r="F10" s="9">
         <v>500</v>
       </c>
       <c r="G10" s="8"/>
-      <c r="H10" s="7">
+      <c r="H10" s="9">
         <v>750</v>
       </c>
       <c r="I10" s="8"/>
-      <c r="J10" s="7">
+      <c r="J10" s="9">
         <v>1000</v>
       </c>
       <c r="K10" s="8"/>
       <c r="M10" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="N10" s="9">
+      <c r="N10" s="7">
         <v>100</v>
       </c>
       <c r="O10" s="8"/>
-      <c r="P10" s="7">
+      <c r="P10" s="9">
         <v>250</v>
       </c>
       <c r="Q10" s="8"/>
-      <c r="R10" s="7">
+      <c r="R10" s="9">
         <v>500</v>
       </c>
       <c r="S10" s="8"/>
-      <c r="T10" s="7">
+      <c r="T10" s="9">
         <v>750</v>
       </c>
       <c r="U10" s="8"/>
-      <c r="V10" s="7">
+      <c r="V10" s="9">
         <v>1000</v>
       </c>
       <c r="W10" s="8"/>
@@ -2138,7 +2132,7 @@
       <c r="J37" s="6">
         <v>2777384</v>
       </c>
-      <c r="K37" s="10">
+      <c r="K37" s="6">
         <v>170445824</v>
       </c>
       <c r="L37" s="6" t="s">
@@ -2463,15 +2457,15 @@
       <c r="A57" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B57" s="9">
+      <c r="B57" s="7">
         <v>1000</v>
       </c>
       <c r="C57" s="8"/>
-      <c r="D57" s="7">
+      <c r="D57" s="9">
         <v>10000</v>
       </c>
       <c r="E57" s="8"/>
-      <c r="F57" s="7">
+      <c r="F57" s="9">
         <v>1000000</v>
       </c>
       <c r="G57" s="8"/>
@@ -2623,15 +2617,15 @@
       <c r="A66" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B66" s="9">
+      <c r="B66" s="7">
         <v>1000</v>
       </c>
       <c r="C66" s="8"/>
-      <c r="D66" s="7">
+      <c r="D66" s="9">
         <v>10000</v>
       </c>
       <c r="E66" s="8"/>
-      <c r="F66" s="7">
+      <c r="F66" s="9">
         <v>1000000</v>
       </c>
       <c r="G66" s="8"/>
@@ -2776,12 +2770,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="D66:E66"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="F57:G57"/>
     <mergeCell ref="P10:Q10"/>
     <mergeCell ref="R10:S10"/>
     <mergeCell ref="T10:U10"/>
@@ -2792,6 +2780,12 @@
     <mergeCell ref="H10:I10"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="N10:O10"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="D66:E66"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="D57:E57"/>
+    <mergeCell ref="F57:G57"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>